<commit_message>
Updated POL_grids_kan50 model - 2026-09-06 23:46
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13964169-BCB8-4254-A000-ECC0F3306E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D6510B1-14B4-479B-9ED5-B56F14EEF0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -544,52 +544,52 @@
     <t>e_demand,ev_battery,H2prd_Elc_PEM,H2prd_Elc_ALK</t>
   </si>
   <si>
+    <t>OstrowiecSwietokrz_POL</t>
+  </si>
+  <si>
+    <t>at grid node - OstrowiecSwietokrz_POL</t>
+  </si>
+  <si>
     <t>Kielce_POL</t>
   </si>
   <si>
     <t>at grid node - Kielce_POL</t>
   </si>
   <si>
+    <t>Zamosc_POL</t>
+  </si>
+  <si>
+    <t>at grid node - Zamosc_POL</t>
+  </si>
+  <si>
     <t>Elk_POL</t>
   </si>
   <si>
     <t>at grid node - Elk_POL</t>
   </si>
   <si>
+    <t>Legnica_POL</t>
+  </si>
+  <si>
+    <t>at grid node - Legnica_POL</t>
+  </si>
+  <si>
+    <t>Olsztyn_POL</t>
+  </si>
+  <si>
+    <t>at grid node - Olsztyn_POL</t>
+  </si>
+  <si>
+    <t>Chelm_POL</t>
+  </si>
+  <si>
+    <t>at grid node - Chelm_POL</t>
+  </si>
+  <si>
     <t>Slupsk_POL</t>
   </si>
   <si>
     <t>at grid node - Slupsk_POL</t>
-  </si>
-  <si>
-    <t>Legnica_POL</t>
-  </si>
-  <si>
-    <t>at grid node - Legnica_POL</t>
-  </si>
-  <si>
-    <t>OstrowiecSwietokrz_POL</t>
-  </si>
-  <si>
-    <t>at grid node - OstrowiecSwietokrz_POL</t>
-  </si>
-  <si>
-    <t>Olsztyn_POL</t>
-  </si>
-  <si>
-    <t>at grid node - Olsztyn_POL</t>
-  </si>
-  <si>
-    <t>Zamosc_POL</t>
-  </si>
-  <si>
-    <t>at grid node - Zamosc_POL</t>
-  </si>
-  <si>
-    <t>Chelm_POL</t>
-  </si>
-  <si>
-    <t>at grid node - Chelm_POL</t>
   </si>
   <si>
     <t>Grajewo_POL</t>
@@ -1102,10 +1102,10 @@
         <v>86</v>
       </c>
       <c r="M11" t="s">
-        <v>102</v>
+        <v>159</v>
       </c>
       <c r="N11" t="s">
-        <v>103</v>
+        <v>160</v>
       </c>
       <c r="O11" t="s">
         <v>167</v>
@@ -1164,10 +1164,10 @@
         <v>86</v>
       </c>
       <c r="M12" t="s">
-        <v>165</v>
+        <v>118</v>
       </c>
       <c r="N12" t="s">
-        <v>166</v>
+        <v>119</v>
       </c>
       <c r="O12" t="s">
         <v>167</v>
@@ -1226,10 +1226,10 @@
         <v>86</v>
       </c>
       <c r="M13" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
       <c r="N13" t="s">
-        <v>143</v>
+        <v>169</v>
       </c>
       <c r="O13" t="s">
         <v>167</v>
@@ -1288,10 +1288,10 @@
         <v>86</v>
       </c>
       <c r="M14" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="N14" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="O14" t="s">
         <v>167</v>
@@ -1350,10 +1350,10 @@
         <v>86</v>
       </c>
       <c r="M15" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="N15" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="O15" t="s">
         <v>167</v>
@@ -1412,10 +1412,10 @@
         <v>86</v>
       </c>
       <c r="M16" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
       <c r="N16" t="s">
-        <v>141</v>
+        <v>95</v>
       </c>
       <c r="O16" t="s">
         <v>167</v>
@@ -1474,10 +1474,10 @@
         <v>86</v>
       </c>
       <c r="M17" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="N17" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="O17" t="s">
         <v>167</v>
@@ -1536,10 +1536,10 @@
         <v>86</v>
       </c>
       <c r="M18" t="s">
-        <v>170</v>
+        <v>112</v>
       </c>
       <c r="N18" t="s">
-        <v>171</v>
+        <v>113</v>
       </c>
       <c r="O18" t="s">
         <v>167</v>
@@ -1598,10 +1598,10 @@
         <v>86</v>
       </c>
       <c r="M19" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="N19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="O19" t="s">
         <v>167</v>
@@ -1660,10 +1660,10 @@
         <v>86</v>
       </c>
       <c r="M20" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="N20" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="O20" t="s">
         <v>167</v>
@@ -1722,10 +1722,10 @@
         <v>86</v>
       </c>
       <c r="M21" t="s">
-        <v>161</v>
+        <v>120</v>
       </c>
       <c r="N21" t="s">
-        <v>162</v>
+        <v>121</v>
       </c>
       <c r="O21" t="s">
         <v>167</v>
@@ -1784,10 +1784,10 @@
         <v>86</v>
       </c>
       <c r="M22" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="N22" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="O22" t="s">
         <v>167</v>
@@ -1846,10 +1846,10 @@
         <v>86</v>
       </c>
       <c r="M23" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="N23" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="O23" t="s">
         <v>167</v>
@@ -1908,10 +1908,10 @@
         <v>86</v>
       </c>
       <c r="M24" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="N24" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="O24" t="s">
         <v>167</v>
@@ -1970,10 +1970,10 @@
         <v>86</v>
       </c>
       <c r="M25" t="s">
-        <v>90</v>
+        <v>146</v>
       </c>
       <c r="N25" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
       <c r="O25" t="s">
         <v>167</v>
@@ -2032,10 +2032,10 @@
         <v>86</v>
       </c>
       <c r="M26" t="s">
-        <v>108</v>
+        <v>170</v>
       </c>
       <c r="N26" t="s">
-        <v>109</v>
+        <v>171</v>
       </c>
       <c r="O26" t="s">
         <v>167</v>
@@ -2094,10 +2094,10 @@
         <v>86</v>
       </c>
       <c r="M27" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
       <c r="N27" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="O27" t="s">
         <v>167</v>
@@ -2156,10 +2156,10 @@
         <v>86</v>
       </c>
       <c r="M28" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="N28" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="O28" t="s">
         <v>167</v>
@@ -2218,10 +2218,10 @@
         <v>86</v>
       </c>
       <c r="M29" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="N29" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="O29" t="s">
         <v>167</v>
@@ -2280,10 +2280,10 @@
         <v>86</v>
       </c>
       <c r="M30" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="N30" t="s">
-        <v>173</v>
+        <v>117</v>
       </c>
       <c r="O30" t="s">
         <v>167</v>
@@ -2342,10 +2342,10 @@
         <v>86</v>
       </c>
       <c r="M31" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="N31" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="O31" t="s">
         <v>167</v>
@@ -2404,10 +2404,10 @@
         <v>86</v>
       </c>
       <c r="M32" t="s">
-        <v>174</v>
+        <v>130</v>
       </c>
       <c r="N32" t="s">
-        <v>175</v>
+        <v>131</v>
       </c>
       <c r="O32" t="s">
         <v>167</v>
@@ -2466,10 +2466,10 @@
         <v>86</v>
       </c>
       <c r="M33" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="N33" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="O33" t="s">
         <v>167</v>
@@ -2528,10 +2528,10 @@
         <v>86</v>
       </c>
       <c r="M34" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="N34" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="O34" t="s">
         <v>167</v>
@@ -2590,10 +2590,10 @@
         <v>86</v>
       </c>
       <c r="M35" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="N35" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="O35" t="s">
         <v>167</v>
@@ -2652,10 +2652,10 @@
         <v>86</v>
       </c>
       <c r="M36" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="N36" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="O36" t="s">
         <v>167</v>
@@ -2714,10 +2714,10 @@
         <v>86</v>
       </c>
       <c r="M37" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="N37" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
       <c r="O37" t="s">
         <v>167</v>
@@ -2776,10 +2776,10 @@
         <v>86</v>
       </c>
       <c r="M38" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="N38" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="O38" t="s">
         <v>167</v>
@@ -2838,10 +2838,10 @@
         <v>86</v>
       </c>
       <c r="M39" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="N39" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="O39" t="s">
         <v>167</v>
@@ -2900,10 +2900,10 @@
         <v>86</v>
       </c>
       <c r="M40" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="N40" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="O40" t="s">
         <v>167</v>
@@ -2938,10 +2938,10 @@
         <v>86</v>
       </c>
       <c r="M41" t="s">
-        <v>124</v>
+        <v>96</v>
       </c>
       <c r="N41" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="O41" t="s">
         <v>167</v>
@@ -2976,10 +2976,10 @@
         <v>86</v>
       </c>
       <c r="M42" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="N42" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="O42" t="s">
         <v>167</v>
@@ -3014,10 +3014,10 @@
         <v>86</v>
       </c>
       <c r="M43" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
       <c r="N43" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="O43" t="s">
         <v>167</v>
@@ -3040,10 +3040,10 @@
         <v>86</v>
       </c>
       <c r="M44" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="N44" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="O44" t="s">
         <v>167</v>
@@ -3066,10 +3066,10 @@
         <v>86</v>
       </c>
       <c r="M45" t="s">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="N45" t="s">
-        <v>105</v>
+        <v>177</v>
       </c>
       <c r="O45" t="s">
         <v>167</v>
@@ -3092,10 +3092,10 @@
         <v>86</v>
       </c>
       <c r="M46" t="s">
-        <v>122</v>
+        <v>87</v>
       </c>
       <c r="N46" t="s">
-        <v>123</v>
+        <v>88</v>
       </c>
       <c r="O46" t="s">
         <v>167</v>
@@ -3118,10 +3118,10 @@
         <v>86</v>
       </c>
       <c r="M47" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="N47" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O47" t="s">
         <v>167</v>
@@ -3144,10 +3144,10 @@
         <v>86</v>
       </c>
       <c r="M48" t="s">
-        <v>180</v>
+        <v>110</v>
       </c>
       <c r="N48" t="s">
-        <v>181</v>
+        <v>111</v>
       </c>
       <c r="O48" t="s">
         <v>167</v>
@@ -3170,10 +3170,10 @@
         <v>86</v>
       </c>
       <c r="M49" t="s">
-        <v>182</v>
+        <v>102</v>
       </c>
       <c r="N49" t="s">
-        <v>183</v>
+        <v>103</v>
       </c>
       <c r="O49" t="s">
         <v>167</v>
@@ -3184,10 +3184,10 @@
         <v>86</v>
       </c>
       <c r="M50" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="N50" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="O50" t="s">
         <v>167</v>
@@ -3198,10 +3198,10 @@
         <v>86</v>
       </c>
       <c r="M51" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="N51" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="O51" t="s">
         <v>167</v>
@@ -3212,10 +3212,10 @@
         <v>86</v>
       </c>
       <c r="M52" t="s">
-        <v>114</v>
+        <v>150</v>
       </c>
       <c r="N52" t="s">
-        <v>115</v>
+        <v>151</v>
       </c>
       <c r="O52" t="s">
         <v>167</v>
@@ -3226,10 +3226,10 @@
         <v>86</v>
       </c>
       <c r="M53" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="N53" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="O53" t="s">
         <v>167</v>
@@ -3240,10 +3240,10 @@
         <v>86</v>
       </c>
       <c r="M54" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="N54" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="O54" t="s">
         <v>167</v>
@@ -3254,10 +3254,10 @@
         <v>86</v>
       </c>
       <c r="M55" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="N55" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="O55" t="s">
         <v>167</v>
@@ -3268,10 +3268,10 @@
         <v>86</v>
       </c>
       <c r="M56" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="N56" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="O56" t="s">
         <v>167</v>
@@ -3282,10 +3282,10 @@
         <v>86</v>
       </c>
       <c r="M57" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="N57" t="s">
-        <v>127</v>
+        <v>183</v>
       </c>
       <c r="O57" t="s">
         <v>167</v>
@@ -3296,10 +3296,10 @@
         <v>86</v>
       </c>
       <c r="M58" t="s">
-        <v>106</v>
+        <v>184</v>
       </c>
       <c r="N58" t="s">
-        <v>107</v>
+        <v>185</v>
       </c>
       <c r="O58" t="s">
         <v>167</v>

</xml_diff>